<commit_message>
feat: compare monthly revenue budget with actuals
</commit_message>
<xml_diff>
--- a/public/financial-template.xlsx
+++ b/public/financial-template.xlsx
@@ -32,6 +32,9 @@
   </si>
   <si>
     <t>Tax</t>
+  </si>
+  <si>
+    <t>RevenueBudget</t>
   </si>
   <si>
     <t>2026-01</t>
@@ -99,10 +102,13 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2">
         <v>182000</v>
@@ -119,10 +125,13 @@
       <c r="F2">
         <v>10000</v>
       </c>
+      <c r="G2">
+        <v>180000</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3">
         <v>198000</v>
@@ -139,10 +148,13 @@
       <c r="F3">
         <v>12000</v>
       </c>
+      <c r="G3">
+        <v>205000</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4">
         <v>191000</v>
@@ -159,6 +171,9 @@
       <c r="F4">
         <v>11000</v>
       </c>
+      <c r="G4">
+        <v>200000</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
Add optional monthly COGS budget variance
</commit_message>
<xml_diff>
--- a/public/financial-template.xlsx
+++ b/public/financial-template.xlsx
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t>RevenueBudget</t>
+  </si>
+  <si>
+    <t>COGSBudget</t>
   </si>
   <si>
     <t>2026-01</t>
@@ -105,10 +108,13 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2">
         <v>182000</v>
@@ -128,10 +134,13 @@
       <c r="G2">
         <v>180000</v>
       </c>
+      <c r="H2">
+        <v>80000</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3">
         <v>198000</v>
@@ -151,10 +160,13 @@
       <c r="G3">
         <v>205000</v>
       </c>
+      <c r="H3">
+        <v>79000</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>191000</v>
@@ -174,6 +186,9 @@
       <c r="G4">
         <v>200000</v>
       </c>
+      <c r="H4">
+        <v>79000</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
Add overall monthly break-even analysis
</commit_message>
<xml_diff>
--- a/public/financial-template.xlsx
+++ b/public/financial-template.xlsx
@@ -38,6 +38,12 @@
   </si>
   <si>
     <t>COGSBudget</t>
+  </si>
+  <si>
+    <t>FixedCosts</t>
+  </si>
+  <si>
+    <t>VariableCosts</t>
   </si>
   <si>
     <t>2026-01</t>
@@ -111,10 +117,16 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2">
         <v>182000</v>
@@ -137,10 +149,16 @@
       <c r="H2">
         <v>80000</v>
       </c>
+      <c r="I2">
+        <v>64000</v>
+      </c>
+      <c r="J2">
+        <v>78000</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>198000</v>
@@ -163,10 +181,16 @@
       <c r="H3">
         <v>79000</v>
       </c>
+      <c r="I3">
+        <v>66000</v>
+      </c>
+      <c r="J3">
+        <v>83000</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B4">
         <v>191000</v>
@@ -188,6 +212,12 @@
       </c>
       <c r="H4">
         <v>79000</v>
+      </c>
+      <c r="I4">
+        <v>65000</v>
+      </c>
+      <c r="J4">
+        <v>81000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>